<commit_message>
Results: Reruns für fehlerhafte Metriken + Selektive Evaluation angepasst
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Backup/gpt_reranking_40_voyage/run_2/ragas_results_20260123_180724.xlsx
+++ b/src/evaluation/data/Backup/gpt_reranking_40_voyage/run_2/ragas_results_20260123_180724.xlsx
@@ -5,17 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\Backup\gpt_reranking_40\run_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\Backup\gpt_reranking_40_voyage\run_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A6FB64-30E7-4EBA-88DD-C617E43C2C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E7B7EA-074A-4CE0-AE2C-86E36F51FAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detaillierte Ergebnisse" sheetId="1" r:id="rId1"/>
     <sheet name="Zusammenfassung" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detaillierte Ergebnisse'!$A$1:$AA$117</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -4433,6 +4436,9 @@
       <c r="M24">
         <v>0.68881467319363776</v>
       </c>
+      <c r="N24">
+        <v>0.99999999750000002</v>
+      </c>
       <c r="O24">
         <v>0</v>
       </c>
@@ -8746,6 +8752,9 @@
       <c r="M76">
         <v>0.69699882813638259</v>
       </c>
+      <c r="N76">
+        <v>0.61538461491124252</v>
+      </c>
       <c r="O76">
         <v>0</v>
       </c>
@@ -10655,6 +10664,9 @@
       <c r="N99">
         <v>0</v>
       </c>
+      <c r="O99">
+        <v>0</v>
+      </c>
       <c r="P99">
         <v>0.1447845995426178</v>
       </c>
@@ -10720,12 +10732,23 @@
       <c r="I100" t="s">
         <v>69</v>
       </c>
-      <c r="J100" s="4"/>
+      <c r="J100" s="5">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="K100">
+        <v>0.75</v>
+      </c>
+      <c r="L100">
+        <v>0.8666666666377778</v>
+      </c>
       <c r="M100">
         <v>0.78463191969742963</v>
       </c>
+      <c r="N100">
+        <v>0.45454545413223141</v>
+      </c>
       <c r="O100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P100">
         <v>0.24941571056842801</v>
@@ -12176,6 +12199,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AA117" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12219,7 +12243,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="5">
-        <v>0.72975205243747432</v>
+        <v>0.72920821290496773</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -12227,7 +12251,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="5">
-        <v>0.79826086956521736</v>
+        <v>0.79784482758620701</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -12235,7 +12259,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>0.82485507243159484</v>
+        <v>0.82521551720923469</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -12243,7 +12267,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="5">
-        <v>0.77957780726490133</v>
+        <v>0.77957780726490122</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -12251,7 +12275,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="4">
-        <v>0.31657489106817821</v>
+        <v>0.32623183411420348</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -12259,7 +12283,7 @@
         <v>14</v>
       </c>
       <c r="B9" s="5">
-        <v>0.60545801124396992</v>
+        <v>0.60885923528497021</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>